<commit_message>
Record protected vehicle data baseline and confirmed tyre width
</commit_message>
<xml_diff>
--- a/Geometry_updated/input/FSAE_VD_3_KASAR .xlsx
+++ b/Geometry_updated/input/FSAE_VD_3_KASAR .xlsx
@@ -12022,7 +12022,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>205</v>
+        <v>152.4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Overall tyre section width used for vehicle envelope</t>
+          <t>User-confirmed 152.4 mm; OLD 2 / Analisis OptimumK!C32. Source workbook is not modified.</t>
         </is>
       </c>
     </row>

</xml_diff>